<commit_message>
update to PLEX file naming program
</commit_message>
<xml_diff>
--- a/Plex.xlsx
+++ b/Plex.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -438,84 +438,84 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Moana-s01e01</t>
+          <t>By The Grace of the Gods-s02e01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Moana-s01e02</t>
+          <t>By The Grace of the Gods-s02e02</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Moana-s01e03</t>
+          <t>By The Grace of the Gods-s02e03</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Moana-s01e04</t>
+          <t>By The Grace of the Gods-s02e04</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Moana-s01e05</t>
+          <t>By The Grace of the Gods-s02e05</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Moana-s01e06</t>
+          <t>By The Grace of the Gods-s02e06</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Moana-s01e07</t>
+          <t>By The Grace of the Gods-s02e07</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Moana-s01e08</t>
+          <t>By The Grace of the Gods-s02e08</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Moana-s01e09</t>
+          <t>By The Grace of the Gods-s02e09</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Moana-s01e10</t>
+          <t>By The Grace of the Gods-s02e10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Moana-s01e11</t>
+          <t>By The Grace of the Gods-s02e11</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Moana-s01e12</t>
+          <t>By The Grace of the Gods-s02e12</t>
         </is>
       </c>
     </row>

</xml_diff>